<commit_message>
Actualizacion de la tabla
</commit_message>
<xml_diff>
--- a/Tabla Unificada.xlsx
+++ b/Tabla Unificada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramir\Documents\cursosProgramacion\CursoHTMLyCSS\proyecto_tabla_de_goleadores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C88F7C4-207A-4BCF-9B43-5CC596C40FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E965A0-B90D-41F0-9017-28B8D907D7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AF445C2-E826-4C2B-AB8F-BB9A5EDA96BC}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="107">
   <si>
     <t>Nombre</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Delantero/Medio</t>
   </si>
   <si>
-    <t>Choppa</t>
-  </si>
-  <si>
     <t>Arquero/Delantero</t>
   </si>
   <si>
@@ -66,12 +63,6 @@
     <t>medio</t>
   </si>
   <si>
-    <t>Primo Fabri</t>
-  </si>
-  <si>
-    <t>Ari</t>
-  </si>
-  <si>
     <t>MEDIO</t>
   </si>
   <si>
@@ -87,54 +78,18 @@
     <t>Laureano</t>
   </si>
   <si>
-    <t>Raviol</t>
-  </si>
-  <si>
-    <t>Fabri H agus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pipa </t>
-  </si>
-  <si>
-    <t>Dante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin </t>
-  </si>
-  <si>
     <t>Franco Amigo TOTO</t>
   </si>
   <si>
-    <t xml:space="preserve">Joel </t>
-  </si>
-  <si>
     <t xml:space="preserve">Medio </t>
   </si>
   <si>
     <t>Arquero</t>
   </si>
   <si>
-    <t>Jorge Flores</t>
-  </si>
-  <si>
-    <t>Aldri Romero</t>
-  </si>
-  <si>
     <t>Ezequiel Dugo 🐻</t>
   </si>
   <si>
-    <t>David Magnone</t>
-  </si>
-  <si>
-    <t>Leo Fernandez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agus Moreno </t>
-  </si>
-  <si>
-    <t>Bruno Bareiro</t>
-  </si>
-  <si>
     <t>Emanuel Chura</t>
   </si>
   <si>
@@ -144,75 +99,12 @@
     <t>Ricky Julcarima</t>
   </si>
   <si>
-    <t xml:space="preserve">Lucas Guillo </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ulises Santillan  </t>
-  </si>
-  <si>
-    <t>Thomy Perez</t>
-  </si>
-  <si>
-    <t>Ferry (Porras)</t>
-  </si>
-  <si>
-    <t>Nicolas Flores</t>
-  </si>
-  <si>
-    <t>Tiago Pujia</t>
-  </si>
-  <si>
-    <t>Agus Vasquez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Federico Suriani </t>
-  </si>
-  <si>
-    <t>Gonzalo Roldan</t>
-  </si>
-  <si>
-    <t>Luciano (topo) Santillan</t>
-  </si>
-  <si>
     <t>Alejo Nieva</t>
   </si>
   <si>
-    <t>Monito (Alan Trinidad)</t>
-  </si>
-  <si>
-    <t>Ale (Abraham)</t>
-  </si>
-  <si>
     <t>Abraham Frias</t>
   </si>
   <si>
-    <t>Alan Vicente</t>
-  </si>
-  <si>
-    <t>Manu Gonzalez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brian Elusanse  </t>
-  </si>
-  <si>
-    <t>Nicolas Ares</t>
-  </si>
-  <si>
-    <t>Alex Ruiz</t>
-  </si>
-  <si>
-    <t>Dylan Perez</t>
-  </si>
-  <si>
-    <t>Lautaro Santillan</t>
-  </si>
-  <si>
-    <t>Nacho (Marinño Makishi)</t>
-  </si>
-  <si>
-    <t>Lihuel Alancay</t>
-  </si>
-  <si>
     <t>TOTO</t>
   </si>
   <si>
@@ -222,21 +114,6 @@
     <t xml:space="preserve">Denber </t>
   </si>
   <si>
-    <t xml:space="preserve">Ezequiel Mataglia </t>
-  </si>
-  <si>
-    <t>Flavio Coulleri</t>
-  </si>
-  <si>
-    <t>Santiago Sanchez</t>
-  </si>
-  <si>
-    <t>Tomas Simon</t>
-  </si>
-  <si>
-    <t>Walter (Wally)</t>
-  </si>
-  <si>
     <t>Masche (Nahuel Garcia)</t>
   </si>
   <si>
@@ -249,21 +126,6 @@
     <t>Jeremias Porti</t>
   </si>
   <si>
-    <t>Ema Ceballo</t>
-  </si>
-  <si>
-    <t>Atahualpo Jose Ignacio</t>
-  </si>
-  <si>
-    <t>Milton Aguirre</t>
-  </si>
-  <si>
-    <t>Brian (Capibara)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pablo Battiston </t>
-  </si>
-  <si>
     <t>Maximiliano Paez</t>
   </si>
   <si>
@@ -273,24 +135,12 @@
     <t>Tadeo Pepey</t>
   </si>
   <si>
-    <t>Thiago Celiz</t>
-  </si>
-  <si>
     <t>Arquero/Medio</t>
   </si>
   <si>
-    <t>Diego Ponce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sebastian </t>
-  </si>
-  <si>
     <t>Ezequiel Roses</t>
   </si>
   <si>
-    <t>Lautaro Mundo  🌍</t>
-  </si>
-  <si>
     <t>Gustavo Claros 😈</t>
   </si>
   <si>
@@ -309,18 +159,6 @@
     <t>Ariel Ramos Q 🐉</t>
   </si>
   <si>
-    <t>Elian Lopez 10</t>
-  </si>
-  <si>
-    <t>Mauri Albornoz 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edgar Ibarra </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agustin Di Stabile  </t>
-  </si>
-  <si>
     <t xml:space="preserve">Dami P </t>
   </si>
   <si>
@@ -330,22 +168,187 @@
     <t>Rodri(Amigo nico)</t>
   </si>
   <si>
-    <t xml:space="preserve">Angel Renato Penaranda </t>
-  </si>
-  <si>
-    <t>Lucas Sanchez</t>
-  </si>
-  <si>
-    <t>Rodri Mundo</t>
-  </si>
-  <si>
     <t>posicion</t>
   </si>
   <si>
-    <t xml:space="preserve">Ezequiel Falce </t>
-  </si>
-  <si>
     <t xml:space="preserve">Director tecnico </t>
+  </si>
+  <si>
+    <t>Tesorero</t>
+  </si>
+  <si>
+    <t>Agustin Di Stabile  🐔</t>
+  </si>
+  <si>
+    <t>Jorge Flores 🐔</t>
+  </si>
+  <si>
+    <t>Edgar Ibarra 🐔</t>
+  </si>
+  <si>
+    <t>Aldri Romero 🐔</t>
+  </si>
+  <si>
+    <t>Nicolas Ares 🏰</t>
+  </si>
+  <si>
+    <t>Choppa 🏰</t>
+  </si>
+  <si>
+    <t>Elian Lopez 🐔</t>
+  </si>
+  <si>
+    <t>Atahualpo Jose Ignacio 🐔</t>
+  </si>
+  <si>
+    <t>David Magnone  🔴⚫️</t>
+  </si>
+  <si>
+    <t>Diego Ponce 🐖</t>
+  </si>
+  <si>
+    <t>Mauri Albornoz 🐖</t>
+  </si>
+  <si>
+    <t>Agus Moreno 🐔</t>
+  </si>
+  <si>
+    <t>Leo Fernandez 🐔</t>
+  </si>
+  <si>
+    <t>Lucas Guillo  🐔</t>
+  </si>
+  <si>
+    <t>Ulises Santillan  🐔</t>
+  </si>
+  <si>
+    <t>Bruno Bareiro🐔</t>
+  </si>
+  <si>
+    <t>Monito (Alan Trinidad) 🐒</t>
+  </si>
+  <si>
+    <t>Ferry (Porras) 🐔</t>
+  </si>
+  <si>
+    <t>Ale (Abraham) 🐔</t>
+  </si>
+  <si>
+    <t>Valen Valenzuela 🐔</t>
+  </si>
+  <si>
+    <t>Thomy Perez 🐔</t>
+  </si>
+  <si>
+    <t>Luciano (topo) Santillan 👹</t>
+  </si>
+  <si>
+    <t>Agus Vasquez 🐖</t>
+  </si>
+  <si>
+    <t>Sebastian 🐔</t>
+  </si>
+  <si>
+    <t>Lucas Sanchez 🐔</t>
+  </si>
+  <si>
+    <t>Angel Renato Penaranda 🐔</t>
+  </si>
+  <si>
+    <t>Federico Suriani 🐔</t>
+  </si>
+  <si>
+    <t>Alex Ruiz 🐔</t>
+  </si>
+  <si>
+    <t>Gonzalo Roldan 🐦‍⬛</t>
+  </si>
+  <si>
+    <t>Nicolas Flores 🐖</t>
+  </si>
+  <si>
+    <t>Nicolas pioli 🐖</t>
+  </si>
+  <si>
+    <t>Rodri Mundo 🐖</t>
+  </si>
+  <si>
+    <t>Pablo Battiston  🐖</t>
+  </si>
+  <si>
+    <t>Ari (Amigo gonza)🐖</t>
+  </si>
+  <si>
+    <t>Brian Elusanse  🐔</t>
+  </si>
+  <si>
+    <t>Nacho (Marinño Makishi) 🐔</t>
+  </si>
+  <si>
+    <t>Kevin 🐔</t>
+  </si>
+  <si>
+    <t>Joel  🐔</t>
+  </si>
+  <si>
+    <t>Brian (Capibara) 🐔</t>
+  </si>
+  <si>
+    <t>Fabri Valenzuela 🐔</t>
+  </si>
+  <si>
+    <t>Dylan Perez 🐔</t>
+  </si>
+  <si>
+    <t>Lautaro Mundo  🌍🐖</t>
+  </si>
+  <si>
+    <t>Milton Aguirre 🐔</t>
+  </si>
+  <si>
+    <t>Ezequiel Falce 🐔</t>
+  </si>
+  <si>
+    <t>Raviol 🐔</t>
+  </si>
+  <si>
+    <t>Tomas Simon 🐔</t>
+  </si>
+  <si>
+    <t>Ema Ceballo 🐔</t>
+  </si>
+  <si>
+    <t>Pipa 🐔</t>
+  </si>
+  <si>
+    <t>Lihuel Alancay 🐔</t>
+  </si>
+  <si>
+    <t>Thiago Celiz 🐂</t>
+  </si>
+  <si>
+    <t>Santiago Sanchez _xDC16_🐖</t>
+  </si>
+  <si>
+    <t>Ezequiel Mataglia _xDC16__xDC16_🐖</t>
+  </si>
+  <si>
+    <t>Fabri H agus 🐖</t>
+  </si>
+  <si>
+    <t>Flavio Coulleri 🐖</t>
+  </si>
+  <si>
+    <t>Tiago Pujia 🦁</t>
+  </si>
+  <si>
+    <t>Lautaro Santillan👹</t>
+  </si>
+  <si>
+    <t>Alan Vicente_xDC79_👹</t>
+  </si>
+  <si>
+    <t>Manu Gonzalez🐔</t>
   </si>
 </sst>
 </file>
@@ -437,12 +440,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,7 +764,7 @@
   <dimension ref="A1:E88"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
+    <col min="1" max="1" width="33.1796875" customWidth="1"/>
     <col min="2" max="2" width="19.26953125" customWidth="1"/>
     <col min="3" max="3" width="14.81640625" customWidth="1"/>
     <col min="4" max="4" width="14.453125" customWidth="1"/>
@@ -781,12 +785,12 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>103</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1">
         <v>33</v>
@@ -804,7 +808,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B3" s="1">
         <v>30</v>
@@ -822,7 +826,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="B4" s="1">
         <v>30</v>
@@ -840,7 +844,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>88</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1">
         <v>25</v>
@@ -858,7 +862,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1">
         <v>20</v>
@@ -876,25 +880,25 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1">
         <v>19</v>
       </c>
       <c r="C7" s="1">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" si="0"/>
-        <v>0.61290322580645162</v>
+        <v>0.59375</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1">
         <v>17</v>
@@ -912,7 +916,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9" s="1">
         <v>17</v>
@@ -930,53 +934,53 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1">
         <v>17</v>
       </c>
       <c r="C10" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" si="0"/>
-        <v>1.4166666666666667</v>
+        <v>1.3076923076923077</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>95</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1">
         <v>16</v>
       </c>
       <c r="C11" s="1">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="1">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="0"/>
-        <v>2.1428571428571428</v>
+        <v>0.8</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>9</v>
@@ -984,7 +988,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="B13" s="1">
         <v>12</v>
@@ -1002,7 +1006,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B14" s="1">
         <v>11</v>
@@ -1020,7 +1024,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="B15" s="1">
         <v>11</v>
@@ -1038,7 +1042,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="B16" s="1">
         <v>10</v>
@@ -1056,7 +1060,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1">
         <v>10</v>
@@ -1074,17 +1078,17 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="B18" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>6</v>
@@ -1092,17 +1096,17 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B19" s="1">
         <v>9</v>
       </c>
       <c r="C19" s="1">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>6</v>
@@ -1110,43 +1114,43 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="B20" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" si="0"/>
-        <v>2.6666666666666665</v>
+        <v>1.2857142857142858</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="B21" s="1">
         <v>8</v>
       </c>
       <c r="C21" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" si="0"/>
-        <v>1.6</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B22" s="1">
         <v>8</v>
@@ -1159,12 +1163,12 @@
         <v>1.6</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="B23" s="1">
         <v>8</v>
@@ -1177,76 +1181,76 @@
         <v>1.3333333333333333</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="B24" s="1">
         <v>8</v>
       </c>
       <c r="C24" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D24" s="1">
         <f t="shared" si="0"/>
-        <v>0.88888888888888884</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="B25" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C25" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B26" s="1">
         <v>7</v>
       </c>
       <c r="C26" s="1">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" si="0"/>
-        <v>0.77777777777777779</v>
+        <v>1.75</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B27" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C27" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>6</v>
@@ -1254,7 +1258,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="B28" s="1">
         <v>6</v>
@@ -1272,17 +1276,17 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="B29" s="1">
         <v>6</v>
       </c>
       <c r="C29" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>6</v>
@@ -1290,17 +1294,17 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B30" s="1">
         <v>6</v>
       </c>
       <c r="C30" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>6</v>
@@ -1308,7 +1312,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="B31" s="1">
         <v>5</v>
@@ -1326,7 +1330,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="B32" s="1">
         <v>5</v>
@@ -1344,17 +1348,17 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="B33" s="1">
         <v>5</v>
       </c>
       <c r="C33" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" si="0"/>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>6</v>
@@ -1362,7 +1366,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="B34" s="1">
         <v>5</v>
@@ -1380,125 +1384,125 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="B35" s="1">
         <v>5</v>
       </c>
       <c r="C35" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" si="1"/>
-        <v>0.83333333333333337</v>
+        <v>1.25</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B36" s="1">
         <v>5</v>
       </c>
       <c r="C36" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" si="1"/>
-        <v>0.7142857142857143</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B37" s="1">
         <v>5</v>
       </c>
       <c r="C37" s="1">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" si="1"/>
-        <v>0.38461538461538464</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="B38" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C38" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" si="1"/>
-        <v>1.3333333333333333</v>
+        <v>0.625</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="B39" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C39" s="1">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="B40" s="1">
         <v>4</v>
       </c>
       <c r="C40" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" si="1"/>
-        <v>0.5714285714285714</v>
+        <v>2</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="B41" s="1">
         <v>4</v>
       </c>
       <c r="C41" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>4</v>
@@ -1506,97 +1510,97 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="B42" s="1">
         <v>4</v>
       </c>
       <c r="C42" s="1">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" si="1"/>
-        <v>0.36363636363636365</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="B43" s="1">
         <v>4</v>
       </c>
       <c r="C43" s="1">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" si="1"/>
-        <v>0.26666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>48</v>
+        <v>103</v>
       </c>
       <c r="B44" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C44" s="1">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="B45" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C45" s="1">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>0.26666666666666666</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="B46" s="1">
         <v>3</v>
       </c>
       <c r="C46" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="B47" s="1">
         <v>3</v>
@@ -1614,43 +1618,43 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="B48" s="1">
         <v>3</v>
       </c>
       <c r="C48" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B49" s="1">
         <v>3</v>
       </c>
       <c r="C49" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="B50" s="1">
         <v>3</v>
@@ -1663,30 +1667,30 @@
         <v>0.5</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="B51" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C51" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="B52" s="1">
         <v>2</v>
@@ -1704,7 +1708,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="B53" s="1">
         <v>2</v>
@@ -1717,12 +1721,12 @@
         <v>2</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B54" s="1">
         <v>2</v>
@@ -1735,12 +1739,12 @@
         <v>2</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="B55" s="1">
         <v>2</v>
@@ -1753,22 +1757,22 @@
         <v>2</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="B56" s="1">
         <v>2</v>
       </c>
       <c r="C56" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D56" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>6</v>
@@ -1776,7 +1780,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="B57" s="1">
         <v>2</v>
@@ -1789,22 +1793,22 @@
         <v>1</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="B58" s="1">
         <v>2</v>
       </c>
       <c r="C58" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D58" s="1">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>4</v>
@@ -1812,7 +1816,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="B59" s="1">
         <v>2</v>
@@ -1825,30 +1829,30 @@
         <v>0.5</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="B60" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D60" s="1">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="B61" s="1">
         <v>1</v>
@@ -1861,12 +1865,12 @@
         <v>1</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="B62" s="1">
         <v>1</v>
@@ -1879,48 +1883,48 @@
         <v>1</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="B63" s="1">
         <v>1</v>
       </c>
       <c r="C63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D63" s="1">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="B64" s="1">
         <v>1</v>
       </c>
       <c r="C64" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64" s="1">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="B65" s="1">
         <v>1</v>
@@ -1938,7 +1942,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
-        <v>21</v>
+        <v>95</v>
       </c>
       <c r="B66" s="1">
         <v>1</v>
@@ -1947,7 +1951,7 @@
         <v>3</v>
       </c>
       <c r="D66" s="1">
-        <f t="shared" ref="D66:D97" si="2">B66/C66</f>
+        <f t="shared" ref="D66:D86" si="2">B66/C66</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="E66" s="1" t="s">
@@ -1956,7 +1960,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="B67" s="1">
         <v>1</v>
@@ -1969,30 +1973,30 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="B68" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C68" s="1">
         <v>3</v>
       </c>
       <c r="D68" s="1">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
-        <v>16</v>
+        <v>102</v>
       </c>
       <c r="B69" s="1">
         <v>0</v>
@@ -2005,12 +2009,12 @@
         <v>0</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="B70" s="1">
         <v>0</v>
@@ -2023,12 +2027,12 @@
         <v>0</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="B71" s="1">
         <v>0</v>
@@ -2041,12 +2045,12 @@
         <v>0</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="B72" s="1">
         <v>0</v>
@@ -2059,30 +2063,30 @@
         <v>0</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B73" s="1">
         <v>0</v>
       </c>
       <c r="C73" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D73" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="B74" s="1">
         <v>0</v>
@@ -2100,7 +2104,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="B75" s="1">
         <v>0</v>
@@ -2113,12 +2117,12 @@
         <v>0</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B76" s="1">
         <v>0</v>
@@ -2131,12 +2135,12 @@
         <v>0</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B77" s="1">
         <v>0</v>
@@ -2149,12 +2153,12 @@
         <v>0</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78" s="4" t="s">
-        <v>99</v>
+      <c r="A78" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="B78" s="1">
         <v>0</v>
@@ -2167,12 +2171,12 @@
         <v>0</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A79" s="1" t="s">
-        <v>102</v>
+      <c r="A79" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="B79" s="1">
         <v>0</v>
@@ -2185,30 +2189,30 @@
         <v>0</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="B80" s="1">
         <v>0</v>
       </c>
       <c r="C80" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="B81" s="1">
         <v>0</v>
@@ -2221,12 +2225,12 @@
         <v>0</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="B82" s="1">
         <v>0</v>
@@ -2239,12 +2243,12 @@
         <v>0</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="B83" s="1">
         <v>0</v>
@@ -2257,12 +2261,12 @@
         <v>0</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="B84" s="1">
         <v>0</v>
@@ -2275,12 +2279,12 @@
         <v>0</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B85" s="1">
         <v>0</v>
@@ -2293,12 +2297,12 @@
         <v>0</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B86" s="1">
         <v>0</v>
@@ -2311,42 +2315,41 @@
         <v>0</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="B87" s="1">
         <v>0</v>
       </c>
       <c r="C87" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D87" s="1">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B88" s="1">
-        <v>0</v>
-      </c>
-      <c r="C88" s="1">
-        <v>0</v>
-      </c>
-      <c r="D88" s="1">
-        <v>0</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>105</v>
+      <c r="A88" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B88" s="5">
+        <v>0</v>
+      </c>
+      <c r="C88" s="5">
+        <v>0</v>
+      </c>
+      <c r="D88" s="5">
+        <v>0</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion de las ultimas dos semanas.
Tema claro y oscuro y una opción de buscar el jugador.
</commit_message>
<xml_diff>
--- a/Tabla Unificada.xlsx
+++ b/Tabla Unificada.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramir\Documents\cursosProgramacion\CursoHTMLyCSS\proyecto_tabla_de_goleadores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03EE3EAB-1C87-4F7F-A961-8D6544B5A911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{540C4462-5857-41E7-87DC-482D2CD49435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AF445C2-E826-4C2B-AB8F-BB9A5EDA96BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="111">
   <si>
     <t>Nombre</t>
   </si>
@@ -135,9 +135,6 @@
     <t>Tadeo Pepey</t>
   </si>
   <si>
-    <t>Arquero/Medio</t>
-  </si>
-  <si>
     <t>Ezequiel Roses</t>
   </si>
   <si>
@@ -355,6 +352,15 @@
   </si>
   <si>
     <t xml:space="preserve">Nehuen </t>
+  </si>
+  <si>
+    <t>vito</t>
+  </si>
+  <si>
+    <t>defensa</t>
+  </si>
+  <si>
+    <t>Franco Ezequiel</t>
   </si>
 </sst>
 </file>
@@ -393,7 +399,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,8 +418,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -436,16 +448,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03004F18-6C3E-4E48-9467-E4389A32EA3B}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.1796875" customWidth="1"/>
@@ -768,6 +795,7 @@
     <col min="3" max="3" width="14.81640625" customWidth="1"/>
     <col min="4" max="4" width="14.453125" customWidth="1"/>
     <col min="5" max="5" width="27.90625" customWidth="1"/>
+    <col min="9" max="9" width="11.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -784,22 +812,22 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C2" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3">
-        <f t="shared" ref="D2:D33" si="0">B2/C2</f>
-        <v>3.4166666666666665</v>
+        <f>B2/C2</f>
+        <v>3.3076923076923075</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>6</v>
@@ -807,35 +835,35 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="B3" s="3">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C3" s="3">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D3" s="3">
-        <f t="shared" si="0"/>
-        <v>5.2857142857142856</v>
+        <f>B3/C3</f>
+        <v>3.4166666666666665</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="3">
         <v>37</v>
       </c>
-      <c r="B4" s="3">
-        <v>33</v>
-      </c>
-      <c r="C4" s="2">
-        <v>9</v>
+      <c r="C4" s="3">
+        <v>7</v>
       </c>
       <c r="D4" s="3">
-        <f t="shared" si="0"/>
-        <v>3.6666666666666665</v>
+        <f>B4/C4</f>
+        <v>5.2857142857142856</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>4</v>
@@ -843,25 +871,25 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B5" s="3">
-        <v>28</v>
-      </c>
-      <c r="C5" s="3">
-        <v>10</v>
+        <v>33</v>
+      </c>
+      <c r="C5" s="2">
+        <v>9</v>
       </c>
       <c r="D5" s="3">
-        <f t="shared" si="0"/>
-        <v>2.8</v>
+        <f>B5/C5</f>
+        <v>3.6666666666666665</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="3">
         <v>25</v>
@@ -870,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="D6" s="3">
-        <f t="shared" si="0"/>
+        <f>B6/C6</f>
         <v>4.166666666666667</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -879,25 +907,25 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="3">
         <v>23</v>
       </c>
       <c r="C7" s="3">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D7" s="3">
-        <f t="shared" si="0"/>
-        <v>0.65714285714285714</v>
+        <f>B7/C7</f>
+        <v>0.6216216216216216</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" s="3">
         <v>20</v>
@@ -906,7 +934,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="3">
-        <f t="shared" si="0"/>
+        <f>B8/C8</f>
         <v>5</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -915,17 +943,17 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" s="3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3">
-        <f t="shared" si="0"/>
-        <v>1.9</v>
+        <f>B9/C9</f>
+        <v>1.8181818181818181</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>8</v>
@@ -933,43 +961,43 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" s="3">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D10" s="3">
-        <f t="shared" si="0"/>
-        <v>2.125</v>
+        <f>B10/C10</f>
+        <v>1.1875</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B11" s="3">
         <v>17</v>
       </c>
       <c r="C11" s="3">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3">
-        <f t="shared" si="0"/>
-        <v>1.1333333333333333</v>
+        <f>B11/C11</f>
+        <v>2.125</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="3">
         <v>16</v>
@@ -978,7 +1006,7 @@
         <v>20</v>
       </c>
       <c r="D12" s="3">
-        <f t="shared" si="0"/>
+        <f>B12/C12</f>
         <v>0.8</v>
       </c>
       <c r="E12" s="3" t="s">
@@ -987,17 +1015,17 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="3">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>B13/C13</f>
+        <v>1.8571428571428572</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>6</v>
@@ -1014,7 +1042,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="3">
-        <f t="shared" si="0"/>
+        <f>B14/C14</f>
         <v>1.8333333333333333</v>
       </c>
       <c r="E14" s="3" t="s">
@@ -1023,7 +1051,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" s="3">
         <v>11</v>
@@ -1032,7 +1060,7 @@
         <v>7</v>
       </c>
       <c r="D15" s="3">
-        <f t="shared" si="0"/>
+        <f>B15/C15</f>
         <v>1.5714285714285714</v>
       </c>
       <c r="E15" s="3" t="s">
@@ -1041,35 +1069,35 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B16" s="3">
+        <v>11</v>
+      </c>
+      <c r="C16" s="3">
+        <v>11</v>
+      </c>
+      <c r="D16" s="3">
+        <f>B16/C16</f>
+        <v>1</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="C16" s="3">
-        <v>7</v>
-      </c>
-      <c r="D16" s="3">
-        <f t="shared" si="0"/>
-        <v>1.4285714285714286</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="B17" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" s="3">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D17" s="3">
-        <f t="shared" si="0"/>
-        <v>1.25</v>
+        <f>B17/C17</f>
+        <v>0.73333333333333328</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>6</v>
@@ -1077,17 +1105,17 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B18" s="3">
         <v>10</v>
       </c>
       <c r="C18" s="3">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D18" s="3">
-        <f t="shared" si="0"/>
-        <v>0.76923076923076927</v>
+        <f>B18/C18</f>
+        <v>1.4285714285714286</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>6</v>
@@ -1095,17 +1123,17 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="B19" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C19" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" si="0"/>
-        <v>1.5</v>
+        <f>B19/C19</f>
+        <v>1.25</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>6</v>
@@ -1113,35 +1141,35 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B20" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C20" s="3">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D20" s="3">
-        <f t="shared" si="0"/>
-        <v>1.2857142857142858</v>
+        <f>B20/C20</f>
+        <v>1</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B21" s="3">
         <v>9</v>
       </c>
       <c r="C21" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D21" s="3">
-        <f t="shared" si="0"/>
-        <v>1.125</v>
+        <f>B21/C21</f>
+        <v>1.5</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -1149,53 +1177,53 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B22" s="3">
         <v>9</v>
       </c>
       <c r="C22" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D22" s="3">
-        <f t="shared" si="0"/>
-        <v>1.125</v>
+        <f>B22/C22</f>
+        <v>1.2857142857142858</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B23" s="3">
         <v>9</v>
       </c>
       <c r="C23" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D23" s="3">
-        <f t="shared" si="0"/>
-        <v>0.9</v>
+        <f>B23/C23</f>
+        <v>1.125</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B24" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" s="3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D24" s="3">
-        <f t="shared" si="0"/>
-        <v>2.6666666666666665</v>
+        <f>B24/C24</f>
+        <v>0.9</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>9</v>
@@ -1203,35 +1231,35 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B25" s="3">
         <v>8</v>
       </c>
       <c r="C25" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D25" s="3">
-        <f t="shared" si="0"/>
-        <v>1.6</v>
+        <f>B25/C25</f>
+        <v>2.6666666666666665</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="B26" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C26" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D26" s="3">
-        <f t="shared" si="0"/>
-        <v>1.75</v>
+        <f>B26/C26</f>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>4</v>
@@ -1239,35 +1267,35 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="B27" s="3">
         <v>7</v>
       </c>
       <c r="C27" s="3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D27" s="3">
-        <f t="shared" si="0"/>
-        <v>0.77777777777777779</v>
+        <f>B27/C27</f>
+        <v>1.75</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="B28" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C28" s="3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D28" s="3">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>B28/C28</f>
+        <v>0.77777777777777779</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>6</v>
@@ -1275,35 +1303,35 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B29" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C29" s="3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D29" s="3">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>B29/C29</f>
+        <v>0.7</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="B30" s="3">
         <v>6</v>
       </c>
       <c r="C30" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D30" s="3">
-        <f t="shared" si="0"/>
-        <v>1.5</v>
+        <f>B30/C30</f>
+        <v>3</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>6</v>
@@ -1311,43 +1339,43 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
       </c>
       <c r="C31" s="3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D31" s="3">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
+        <f>B31/C31</f>
+        <v>3</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D32" s="3">
-        <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
+        <f>B32/C32</f>
+        <v>1.5</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="3">
         <v>5</v>
@@ -1356,7 +1384,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="3">
-        <f t="shared" si="0"/>
+        <f>B33/C33</f>
         <v>5</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -1365,7 +1393,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B34" s="3">
         <v>5</v>
@@ -1374,7 +1402,7 @@
         <v>1</v>
       </c>
       <c r="D34" s="3">
-        <f t="shared" ref="D34:D65" si="1">B34/C34</f>
+        <f>B34/C34</f>
         <v>5</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -1383,7 +1411,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B35" s="3">
         <v>5</v>
@@ -1392,7 +1420,7 @@
         <v>2</v>
       </c>
       <c r="D35" s="3">
-        <f t="shared" si="1"/>
+        <f>B35/C35</f>
         <v>2.5</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -1401,7 +1429,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B36" s="3">
         <v>5</v>
@@ -1410,7 +1438,7 @@
         <v>4</v>
       </c>
       <c r="D36" s="3">
-        <f t="shared" si="1"/>
+        <f>B36/C36</f>
         <v>1.25</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -1419,7 +1447,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B37" s="3">
         <v>5</v>
@@ -1428,7 +1456,7 @@
         <v>4</v>
       </c>
       <c r="D37" s="3">
-        <f t="shared" si="1"/>
+        <f>B37/C37</f>
         <v>1.25</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -1437,43 +1465,43 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B38" s="3">
         <v>5</v>
       </c>
       <c r="C38" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D38" s="3">
-        <f t="shared" si="1"/>
-        <v>0.83333333333333337</v>
+        <f>B38/C38</f>
+        <v>1.25</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="B39" s="3">
         <v>5</v>
       </c>
       <c r="C39" s="3">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D39" s="3">
-        <f t="shared" si="1"/>
-        <v>0.38461538461538464</v>
+        <f>B39/C39</f>
+        <v>0.83333333333333337</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B40" s="3">
         <v>5</v>
@@ -1482,7 +1510,7 @@
         <v>14</v>
       </c>
       <c r="D40" s="3">
-        <f t="shared" si="1"/>
+        <f>B40/C40</f>
         <v>0.35714285714285715</v>
       </c>
       <c r="E40" s="3" t="s">
@@ -1491,20 +1519,20 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B41" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C41" s="3">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D41" s="3">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>B41/C41</f>
+        <v>0.35714285714285715</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
@@ -1518,7 +1546,7 @@
         <v>3</v>
       </c>
       <c r="D42" s="3">
-        <f t="shared" si="1"/>
+        <f>B42/C42</f>
         <v>1.3333333333333333</v>
       </c>
       <c r="E42" s="3" t="s">
@@ -1527,7 +1555,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B43" s="3">
         <v>4</v>
@@ -1536,7 +1564,7 @@
         <v>6</v>
       </c>
       <c r="D43" s="3">
-        <f t="shared" si="1"/>
+        <f>B43/C43</f>
         <v>0.66666666666666663</v>
       </c>
       <c r="E43" s="3" t="s">
@@ -1545,7 +1573,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B44" s="3">
         <v>4</v>
@@ -1554,7 +1582,7 @@
         <v>8</v>
       </c>
       <c r="D44" s="3">
-        <f t="shared" si="1"/>
+        <f>B44/C44</f>
         <v>0.5</v>
       </c>
       <c r="E44" s="3" t="s">
@@ -1563,7 +1591,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B45" s="3">
         <v>4</v>
@@ -1572,7 +1600,7 @@
         <v>17</v>
       </c>
       <c r="D45" s="3">
-        <f t="shared" si="1"/>
+        <f>B45/C45</f>
         <v>0.23529411764705882</v>
       </c>
       <c r="E45" s="3" t="s">
@@ -1590,7 +1618,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="3">
-        <f t="shared" si="1"/>
+        <f>B46/C46</f>
         <v>3</v>
       </c>
       <c r="E46" s="3" t="s">
@@ -1599,17 +1627,17 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B47" s="3">
         <v>3</v>
       </c>
       <c r="C47" s="3">
-        <v>2</v>
-      </c>
-      <c r="D47" s="3">
-        <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>1</v>
+      </c>
+      <c r="D47" s="8">
+        <f>B47/C47</f>
+        <v>3</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>4</v>
@@ -1617,7 +1645,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="B48" s="3">
         <v>3</v>
@@ -1626,7 +1654,7 @@
         <v>2</v>
       </c>
       <c r="D48" s="3">
-        <f t="shared" si="1"/>
+        <f>B48/C48</f>
         <v>1.5</v>
       </c>
       <c r="E48" s="3" t="s">
@@ -1635,38 +1663,38 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="B49" s="3">
         <v>3</v>
       </c>
       <c r="C49" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D49" s="3">
-        <f t="shared" si="1"/>
-        <v>0.6</v>
+        <f>B49/C49</f>
+        <v>1.5</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="B50" s="3">
         <v>3</v>
       </c>
       <c r="C50" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D50" s="3">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
+        <f>B50/C50</f>
+        <v>0.6</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
@@ -1677,37 +1705,37 @@
         <v>3</v>
       </c>
       <c r="C51" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" si="1"/>
-        <v>0.375</v>
+        <f>B51/C51</f>
+        <v>0.5</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="B52" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C52" s="3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D52" s="3">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>B52/C52</f>
+        <v>0.375</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B53" s="3">
         <v>2</v>
@@ -1716,7 +1744,7 @@
         <v>1</v>
       </c>
       <c r="D53" s="3">
-        <f t="shared" si="1"/>
+        <f>B53/C53</f>
         <v>2</v>
       </c>
       <c r="E53" s="3" t="s">
@@ -1725,7 +1753,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B54" s="3">
         <v>2</v>
@@ -1734,16 +1762,16 @@
         <v>1</v>
       </c>
       <c r="D54" s="3">
-        <f t="shared" si="1"/>
+        <f>B54/C54</f>
         <v>2</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="B55" s="3">
         <v>2</v>
@@ -1751,17 +1779,17 @@
       <c r="C55" s="3">
         <v>1</v>
       </c>
-      <c r="D55" s="4">
-        <f t="shared" si="1"/>
+      <c r="D55" s="3">
+        <f>B55/C55</f>
         <v>2</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B56" s="3">
         <v>2</v>
@@ -1769,17 +1797,17 @@
       <c r="C56" s="3">
         <v>2</v>
       </c>
-      <c r="D56" s="3">
-        <f t="shared" si="1"/>
+      <c r="D56" s="4">
+        <f>B56/C56</f>
         <v>1</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B57" s="3">
         <v>2</v>
@@ -1788,16 +1816,16 @@
         <v>2</v>
       </c>
       <c r="D57" s="3">
-        <f t="shared" si="1"/>
+        <f>B57/C57</f>
         <v>1</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B58" s="3">
         <v>2</v>
@@ -1806,7 +1834,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="3">
-        <f t="shared" si="1"/>
+        <f>B58/C58</f>
         <v>1</v>
       </c>
       <c r="E58" s="3" t="s">
@@ -1815,7 +1843,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B59" s="3">
         <v>2</v>
@@ -1824,26 +1852,26 @@
         <v>2</v>
       </c>
       <c r="D59" s="3">
-        <f t="shared" si="1"/>
+        <f>B59/C59</f>
         <v>1</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B60" s="3">
         <v>2</v>
       </c>
       <c r="C60" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D60" s="3">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
+        <f>B60/C60</f>
+        <v>1</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>4</v>
@@ -1851,17 +1879,17 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B61" s="3">
         <v>2</v>
       </c>
       <c r="C61" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D61" s="3">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
+        <f>B61/C61</f>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>9</v>
@@ -1869,61 +1897,61 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B62" s="3">
         <v>2</v>
       </c>
       <c r="C62" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" s="3">
-        <f t="shared" si="1"/>
-        <v>0.4</v>
+        <f>B62/C62</f>
+        <v>0.5</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B63" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C63" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D63" s="3">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>B63/C63</f>
+        <v>0.4</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>16</v>
+        <v>94</v>
       </c>
       <c r="B64" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C64" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D64" s="3">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>B64/C64</f>
+        <v>0.4</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="B65" s="3">
         <v>1</v>
@@ -1932,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="3">
-        <f t="shared" si="1"/>
+        <f>B65/C65</f>
         <v>1</v>
       </c>
       <c r="E65" s="3" t="s">
@@ -1941,35 +1969,35 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B66" s="3">
         <v>1</v>
       </c>
       <c r="C66" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D66" s="3">
-        <f t="shared" ref="D66:D97" si="2">B66/C66</f>
-        <v>0.5</v>
+        <f>B66/C66</f>
+        <v>1</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B67" s="3">
         <v>1</v>
       </c>
       <c r="C67" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D67" s="3">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <f>B67/C67</f>
+        <v>1</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>6</v>
@@ -1977,106 +2005,105 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="B68" s="3">
         <v>1</v>
       </c>
       <c r="C68" s="3">
-        <v>3</v>
-      </c>
-      <c r="D68" s="3">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <v>1</v>
+      </c>
+      <c r="D68" s="4">
+        <f>B68/C68</f>
+        <v>1</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>6</v>
+        <v>109</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>101</v>
+        <v>25</v>
       </c>
       <c r="B69" s="3">
         <v>1</v>
       </c>
       <c r="C69" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D69" s="3">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
+        <f>B69/C69</f>
+        <v>0.5</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="B70" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C70" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D70" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>B70/C70</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B71" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C71" s="3">
         <v>3</v>
       </c>
       <c r="D71" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>B71/C71</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="B72" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C72" s="3">
         <v>3</v>
       </c>
       <c r="D72" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>B72/C72</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="B73" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C73" s="3">
         <v>3</v>
       </c>
-      <c r="D73" s="3">
-        <f t="shared" si="2"/>
+      <c r="D73" s="4">
         <v>0</v>
       </c>
       <c r="E73" s="3" t="s">
@@ -2091,28 +2118,28 @@
         <v>0</v>
       </c>
       <c r="C74" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D74" s="3">
-        <f t="shared" si="2"/>
+        <f>B74/C74</f>
         <v>0</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>33</v>
+        <v>101</v>
       </c>
       <c r="B75" s="3">
         <v>0</v>
       </c>
       <c r="C75" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D75" s="3">
-        <f t="shared" si="2"/>
+        <f>B75/C75</f>
         <v>0</v>
       </c>
       <c r="E75" s="3" t="s">
@@ -2121,34 +2148,34 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
-        <v>94</v>
+        <v>13</v>
       </c>
       <c r="B76" s="3">
         <v>0</v>
       </c>
       <c r="C76" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D76" s="3">
-        <f t="shared" si="2"/>
+        <f>B76/C76</f>
         <v>0</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="B77" s="3">
         <v>0</v>
       </c>
       <c r="C77" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D77" s="3">
-        <f t="shared" si="2"/>
+        <f>B77/C77</f>
         <v>0</v>
       </c>
       <c r="E77" s="3" t="s">
@@ -2157,25 +2184,25 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="B78" s="3">
         <v>0</v>
       </c>
       <c r="C78" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D78" s="3">
-        <f t="shared" si="2"/>
+        <f>B78/C78</f>
         <v>0</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B79" s="3">
         <v>0</v>
@@ -2184,16 +2211,16 @@
         <v>2</v>
       </c>
       <c r="D79" s="3">
-        <f t="shared" si="2"/>
+        <f>B79/C79</f>
         <v>0</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="B80" s="3">
         <v>0</v>
@@ -2202,7 +2229,7 @@
         <v>2</v>
       </c>
       <c r="D80" s="3">
-        <f t="shared" si="2"/>
+        <f>B80/C80</f>
         <v>0</v>
       </c>
       <c r="E80" s="3" t="s">
@@ -2211,7 +2238,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="B81" s="3">
         <v>0</v>
@@ -2220,43 +2247,43 @@
         <v>2</v>
       </c>
       <c r="D81" s="3">
-        <f t="shared" si="2"/>
+        <f>B81/C81</f>
         <v>0</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B82" s="3">
         <v>0</v>
       </c>
       <c r="C82" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D82" s="3">
-        <f t="shared" si="2"/>
+        <f>B82/C82</f>
         <v>0</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B83" s="3">
         <v>0</v>
       </c>
       <c r="C83" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="3">
-        <f t="shared" si="2"/>
+        <f>B83/C83</f>
         <v>0</v>
       </c>
       <c r="E83" s="3" t="s">
@@ -2265,25 +2292,25 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="B84" s="3">
         <v>0</v>
       </c>
       <c r="C84" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" s="3">
-        <f t="shared" si="2"/>
+        <f>B84/C84</f>
         <v>0</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="B85" s="3">
         <v>0</v>
@@ -2292,16 +2319,16 @@
         <v>1</v>
       </c>
       <c r="D85" s="3">
-        <f t="shared" si="2"/>
+        <f>B85/C85</f>
         <v>0</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B86" s="3">
         <v>0</v>
@@ -2310,16 +2337,16 @@
         <v>1</v>
       </c>
       <c r="D86" s="3">
-        <f t="shared" si="2"/>
+        <f>B86/C86</f>
         <v>0</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="B87" s="3">
         <v>0</v>
@@ -2328,11 +2355,11 @@
         <v>1</v>
       </c>
       <c r="D87" s="3">
-        <f t="shared" si="2"/>
+        <f>B87/C87</f>
         <v>0</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
@@ -2343,54 +2370,91 @@
         <v>0</v>
       </c>
       <c r="C88" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D88" s="3">
+        <f>B88/C88</f>
         <v>0</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>47</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B89" s="4">
-        <v>0</v>
-      </c>
-      <c r="C89" s="4">
-        <v>0</v>
-      </c>
-      <c r="D89" s="4">
+        <v>34</v>
+      </c>
+      <c r="B89" s="3">
+        <v>0</v>
+      </c>
+      <c r="C89" s="3">
+        <v>1</v>
+      </c>
+      <c r="D89" s="3">
+        <f>B89/C89</f>
         <v>0</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="B90" s="3">
         <v>0</v>
       </c>
       <c r="C90" s="3">
-        <v>0</v>
-      </c>
-      <c r="D90" s="4">
+        <v>1</v>
+      </c>
+      <c r="D90" s="3">
+        <f>B90/C90</f>
         <v>0</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>9</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B91" s="5">
+        <v>0</v>
+      </c>
+      <c r="C91" s="5">
+        <v>0</v>
+      </c>
+      <c r="D91" s="3">
+        <v>0</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B92" s="6">
+        <v>0</v>
+      </c>
+      <c r="C92" s="6">
+        <v>0</v>
+      </c>
+      <c r="D92" s="7">
+        <v>0</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E90">
-    <sortCondition descending="1" ref="B2:B90"/>
-    <sortCondition descending="1" ref="D2:D90"/>
-    <sortCondition descending="1" ref="C2:C90"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E92">
+    <sortCondition descending="1" ref="B2:B92"/>
+    <sortCondition descending="1" ref="D2:D92"/>
+    <sortCondition descending="1" ref="C2:C92"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualizacion de la pagina de goleadores 8/10/2026
</commit_message>
<xml_diff>
--- a/Tabla Unificada.xlsx
+++ b/Tabla Unificada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramir\Documents\cursosProgramacion\CursoHTMLyCSS\proyecto_tabla_de_goleadores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B489578C-232D-468E-B1EC-C2D730B3CC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D1FFA6F-82CC-4492-BC75-6D7B3A2722A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AF445C2-E826-4C2B-AB8F-BB9A5EDA96BC}"/>
   </bookViews>
@@ -363,7 +363,7 @@
     <t>Franco David Chura Calle</t>
   </si>
   <si>
-    <t>Maximo Santillan</t>
+    <t>Maximiliano Santillan</t>
   </si>
 </sst>
 </file>
@@ -800,7 +800,7 @@
     <col min="3" max="3" width="14.81640625" customWidth="1"/>
     <col min="4" max="4" width="14.453125" customWidth="1"/>
     <col min="5" max="5" width="27.90625" customWidth="1"/>
-    <col min="9" max="9" width="11.90625" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -822,17 +822,17 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B2" s="3">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C2" s="3">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" s="3">
         <f>B2/C2</f>
-        <v>3.3076923076923075</v>
+        <v>3.4</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>6</v>
@@ -840,17 +840,17 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C3" s="3">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" s="3">
         <f>B3/C3</f>
-        <v>3.3076923076923075</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>6</v>
@@ -861,14 +861,14 @@
         <v>88</v>
       </c>
       <c r="B4" s="3">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C4" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="3">
         <f>B4/C4</f>
-        <v>5.2857142857142856</v>
+        <v>5.25</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>4</v>
@@ -915,14 +915,14 @@
         <v>39</v>
       </c>
       <c r="B7" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="3">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D7" s="3">
         <f>B7/C7</f>
-        <v>0.60526315789473684</v>
+        <v>0.6</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>18</v>
@@ -954,11 +954,11 @@
         <v>21</v>
       </c>
       <c r="C9" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="3">
         <f>B9/C9</f>
-        <v>1.75</v>
+        <v>1.6153846153846154</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>8</v>
@@ -1038,107 +1038,107 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="B14" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D14" s="3">
         <f>B14/C14</f>
-        <v>1.8333333333333333</v>
+        <v>1.5</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" s="3">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D15" s="3">
         <f>B15/C15</f>
-        <v>1.5714285714285714</v>
+        <v>0.92307692307692313</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B16" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C16" s="3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D16" s="3">
         <f>B16/C16</f>
-        <v>0.91666666666666663</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="B17" s="3">
         <v>11</v>
       </c>
       <c r="C17" s="3">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D17" s="3">
         <f>B17/C17</f>
-        <v>0.6875</v>
+        <v>1.8333333333333333</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18" s="3">
         <v>7</v>
       </c>
       <c r="D18" s="3">
         <f>B18/C18</f>
-        <v>1.4285714285714286</v>
+        <v>1.5714285714285714</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="B19" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C19" s="3">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D19" s="3">
         <f>B19/C19</f>
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>6</v>
@@ -1146,17 +1146,17 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3">
         <v>10</v>
       </c>
       <c r="C20" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D20" s="3">
         <f>B20/C20</f>
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
@@ -1170,11 +1170,11 @@
         <v>9</v>
       </c>
       <c r="C21" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D21" s="3">
         <f>B21/C21</f>
-        <v>1.5</v>
+        <v>1.2857142857142858</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -1224,11 +1224,11 @@
         <v>9</v>
       </c>
       <c r="C24" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D24" s="3">
         <f>B24/C24</f>
-        <v>0.81818181818181823</v>
+        <v>0.75</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>9</v>
@@ -1254,35 +1254,35 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B26" s="3">
         <v>8</v>
       </c>
       <c r="C26" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="3">
         <f>B26/C26</f>
-        <v>1.3333333333333333</v>
+        <v>1.6</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="B27" s="3">
+        <v>8</v>
+      </c>
+      <c r="C27" s="3">
         <v>7</v>
-      </c>
-      <c r="C27" s="3">
-        <v>4</v>
       </c>
       <c r="D27" s="3">
         <f>B27/C27</f>
-        <v>1.75</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>4</v>
@@ -1290,53 +1290,53 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>62</v>
+        <v>109</v>
       </c>
       <c r="B28" s="3">
         <v>7</v>
       </c>
       <c r="C28" s="3">
-        <v>9</v>
-      </c>
-      <c r="D28" s="3">
+        <v>3</v>
+      </c>
+      <c r="D28" s="8">
         <f>B28/C28</f>
-        <v>0.77777777777777779</v>
+        <v>2.3333333333333335</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="B29" s="3">
         <v>7</v>
       </c>
       <c r="C29" s="3">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D29" s="3">
         <f>B29/C29</f>
-        <v>0.7</v>
+        <v>1.75</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B30" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C30" s="3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D30" s="3">
         <f>B30/C30</f>
-        <v>3</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>6</v>
@@ -1344,35 +1344,35 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B31" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31" s="3">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D31" s="3">
         <f>B31/C31</f>
-        <v>3</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="B32" s="3">
         <v>6</v>
       </c>
       <c r="C32" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D32" s="3">
         <f>B32/C32</f>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>6</v>
@@ -1380,35 +1380,35 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B33" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C33" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="3">
         <f>B33/C33</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B34" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D34" s="3">
         <f>B34/C34</f>
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>6</v>
@@ -1416,35 +1416,35 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B35" s="3">
         <v>5</v>
       </c>
       <c r="C35" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="3">
         <f>B35/C35</f>
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="B36" s="3">
         <v>5</v>
       </c>
       <c r="C36" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D36" s="3">
         <f>B36/C36</f>
-        <v>1.25</v>
+        <v>5</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>6</v>
@@ -1452,17 +1452,17 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B37" s="3">
         <v>5</v>
       </c>
       <c r="C37" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" s="3">
         <f>B37/C37</f>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>6</v>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B38" s="3">
         <v>5</v>
@@ -1488,43 +1488,43 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B39" s="3">
         <v>5</v>
       </c>
       <c r="C39" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D39" s="3">
         <f>B39/C39</f>
-        <v>0.83333333333333337</v>
+        <v>1.25</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="B40" s="3">
         <v>5</v>
       </c>
       <c r="C40" s="3">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D40" s="3">
         <f>B40/C40</f>
-        <v>0.35714285714285715</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="B41" s="3">
         <v>5</v>
@@ -1542,20 +1542,20 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="B42" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C42" s="3">
-        <v>2</v>
-      </c>
-      <c r="D42" s="8">
+        <v>14</v>
+      </c>
+      <c r="D42" s="3">
         <f>B42/C42</f>
-        <v>2</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
@@ -1620,11 +1620,11 @@
         <v>4</v>
       </c>
       <c r="C46" s="3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D46" s="3">
         <f>B46/C46</f>
-        <v>0.23529411764705882</v>
+        <v>0.22222222222222221</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>9</v>
@@ -1938,17 +1938,17 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B64" s="3">
         <v>2</v>
       </c>
       <c r="C64" s="3">
-        <v>6</v>
-      </c>
-      <c r="D64" s="3">
+        <v>5</v>
+      </c>
+      <c r="D64" s="4">
         <f>B64/C64</f>
-        <v>0.33333333333333331</v>
+        <v>0.4</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>9</v>
@@ -1956,25 +1956,25 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="B65" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" s="3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D65" s="3">
         <f>B65/C65</f>
-        <v>1</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="B66" s="3">
         <v>1</v>
@@ -1987,12 +1987,12 @@
         <v>1</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="B67" s="3">
         <v>1</v>
@@ -2005,12 +2005,12 @@
         <v>1</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="B68" s="3">
         <v>1</v>
@@ -2018,17 +2018,17 @@
       <c r="C68" s="3">
         <v>1</v>
       </c>
-      <c r="D68" s="4">
+      <c r="D68" s="3">
         <f>B68/C68</f>
         <v>1</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>108</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B69" s="3">
         <v>1</v>
@@ -2036,17 +2036,17 @@
       <c r="C69" s="3">
         <v>1</v>
       </c>
-      <c r="D69" s="9">
+      <c r="D69" s="4">
         <f>B69/C69</f>
         <v>1</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>6</v>
+        <v>108</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
-        <v>25</v>
+        <v>111</v>
       </c>
       <c r="B70" s="3">
         <v>1</v>
@@ -2054,35 +2054,35 @@
       <c r="C70" s="3">
         <v>2</v>
       </c>
-      <c r="D70" s="3">
+      <c r="D70" s="9">
         <f>B70/C70</f>
         <v>0.5</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B71" s="3">
         <v>1</v>
       </c>
       <c r="C71" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D71" s="3">
         <f>B71/C71</f>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
-        <v>94</v>
+        <v>30</v>
       </c>
       <c r="B72" s="3">
         <v>1</v>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B73" s="3">
         <v>1</v>
@@ -2113,21 +2113,22 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="B74" s="3">
         <v>1</v>
       </c>
       <c r="C74" s="3">
-        <v>4</v>
-      </c>
-      <c r="D74" s="4">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="D74" s="3">
+        <f>B74/C74</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>9</v>
@@ -2321,7 +2322,7 @@
         <v>0</v>
       </c>
       <c r="C85" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D85" s="3">
         <f>B85/C85</f>
@@ -2404,20 +2405,20 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="3" t="s">
+      <c r="A90" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B90" s="3">
-        <v>0</v>
-      </c>
-      <c r="C90" s="3">
+      <c r="B90" s="5">
+        <v>0</v>
+      </c>
+      <c r="C90" s="5">
         <v>1</v>
       </c>
       <c r="D90" s="3">
         <f>B90/C90</f>
         <v>0</v>
       </c>
-      <c r="E90" s="3" t="s">
+      <c r="E90" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2431,7 +2432,7 @@
       <c r="C91" s="5">
         <v>1</v>
       </c>
-      <c r="D91" s="3">
+      <c r="D91" s="10">
         <f>B91/C91</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Goles cargados + puskas
</commit_message>
<xml_diff>
--- a/Tabla Unificada.xlsx
+++ b/Tabla Unificada.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramir\Documents\cursosProgramacion\CursoHTMLyCSS\proyecto_tabla_de_goleadores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D1FFA6F-82CC-4492-BC75-6D7B3A2722A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A467DC02-346B-494A-991A-48DE387A2F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AF445C2-E826-4C2B-AB8F-BB9A5EDA96BC}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="113">
   <si>
     <t>Nombre</t>
   </si>
@@ -204,9 +204,6 @@
     <t>Mauri Albornoz 🐖</t>
   </si>
   <si>
-    <t>Agus Moreno 🐔</t>
-  </si>
-  <si>
     <t>Leo Fernandez 🐔</t>
   </si>
   <si>
@@ -364,6 +361,12 @@
   </si>
   <si>
     <t>Maximiliano Santillan</t>
+  </si>
+  <si>
+    <t>Santiago V</t>
+  </si>
+  <si>
+    <t>Agus Moreno 🐔🔪 (BOCA EL MAS GRANDE)</t>
   </si>
 </sst>
 </file>
@@ -493,6 +496,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="⚽">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA62AB00-C3F1-46FE-BB5A-16F389703D53}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8267700" y="184150"/>
+          <a:ext cx="12700" cy="12700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -792,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03004F18-6C3E-4E48-9467-E4389A32EA3B}">
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.1796875" customWidth="1"/>
@@ -858,7 +927,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B4" s="3">
         <v>42</v>
@@ -894,38 +963,38 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="B6" s="3">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="3">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3">
         <f>B6/C6</f>
-        <v>4.166666666666667</v>
+        <v>2.0714285714285716</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B7" s="3">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3">
         <f>B7/C7</f>
-        <v>0.6</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -933,14 +1002,14 @@
         <v>40</v>
       </c>
       <c r="B8" s="3">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="3">
         <f>B8/C8</f>
-        <v>1.2941176470588236</v>
+        <v>1.3888888888888888</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
@@ -948,20 +1017,20 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B9" s="3">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="D9" s="3">
         <f>B9/C9</f>
-        <v>1.6153846153846154</v>
+        <v>0.6097560975609756</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -972,11 +1041,11 @@
         <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D10" s="3">
         <f>B10/C10</f>
-        <v>5</v>
+        <v>1.4285714285714286</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>4</v>
@@ -984,71 +1053,71 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B11" s="3">
         <v>17</v>
       </c>
       <c r="C11" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3">
         <f>B11/C11</f>
-        <v>1.8888888888888888</v>
+        <v>2.125</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B12" s="3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3">
         <f>B12/C12</f>
-        <v>0.8</v>
+        <v>1.8888888888888888</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13" s="3">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C13" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" s="3">
         <f>B13/C13</f>
-        <v>1.625</v>
+        <v>1.7777777777777777</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14" s="3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D14" s="3">
         <f>B14/C14</f>
-        <v>1.5</v>
+        <v>0.78947368421052633</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>6</v>
@@ -1056,38 +1125,38 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B15" s="3">
         <v>12</v>
       </c>
       <c r="C15" s="3">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D15" s="3">
         <f>B15/C15</f>
-        <v>0.92307692307692313</v>
+        <v>1.5</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B16" s="3">
         <v>12</v>
       </c>
       <c r="C16" s="3">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D16" s="3">
         <f>B16/C16</f>
-        <v>0.66666666666666663</v>
+        <v>0.92307692307692313</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1146,35 +1215,35 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="B20" s="3">
         <v>10</v>
       </c>
       <c r="C20" s="3">
-        <v>8</v>
-      </c>
-      <c r="D20" s="3">
+        <v>4</v>
+      </c>
+      <c r="D20" s="8">
         <f>B20/C20</f>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C21" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D21" s="3">
         <f>B21/C21</f>
-        <v>1.2857142857142858</v>
+        <v>1.25</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -1182,7 +1251,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B22" s="3">
         <v>9</v>
@@ -1195,58 +1264,58 @@
         <v>1.2857142857142858</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B23" s="3">
         <v>9</v>
       </c>
       <c r="C23" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D23" s="3">
         <f>B23/C23</f>
-        <v>1.125</v>
+        <v>1.2857142857142858</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B24" s="3">
         <v>9</v>
       </c>
       <c r="C24" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D24" s="3">
         <f>B24/C24</f>
-        <v>0.75</v>
+        <v>1.125</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B25" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C25" s="3">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D25" s="3">
         <f>B25/C25</f>
-        <v>2.6666666666666665</v>
+        <v>0.75</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>9</v>
@@ -1254,53 +1323,53 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="B26" s="3">
         <v>8</v>
       </c>
       <c r="C26" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D26" s="3">
         <f>B26/C26</f>
-        <v>1.6</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B27" s="3">
         <v>8</v>
       </c>
       <c r="C27" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D27" s="3">
         <f>B27/C27</f>
-        <v>1.1428571428571428</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="B28" s="3">
+        <v>8</v>
+      </c>
+      <c r="C28" s="3">
         <v>7</v>
       </c>
-      <c r="C28" s="3">
-        <v>3</v>
-      </c>
-      <c r="D28" s="8">
+      <c r="D28" s="3">
         <f>B28/C28</f>
-        <v>2.3333333333333335</v>
+        <v>1.1428571428571428</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>4</v>
@@ -1326,7 +1395,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B30" s="3">
         <v>7</v>
@@ -1344,7 +1413,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B31" s="3">
         <v>7</v>
@@ -1380,7 +1449,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B33" s="3">
         <v>6</v>
@@ -1398,7 +1467,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B34" s="3">
         <v>6</v>
@@ -1416,7 +1485,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B35" s="3">
         <v>5</v>
@@ -1452,7 +1521,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B37" s="3">
         <v>5</v>
@@ -1470,7 +1539,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B38" s="3">
         <v>5</v>
@@ -1488,7 +1557,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B39" s="3">
         <v>5</v>
@@ -1506,7 +1575,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" s="3">
         <v>5</v>
@@ -1524,7 +1593,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B41" s="3">
         <v>5</v>
@@ -1542,7 +1611,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B42" s="3">
         <v>5</v>
@@ -1560,35 +1629,35 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>24</v>
+        <v>74</v>
       </c>
       <c r="B43" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C43" s="3">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="D43" s="3">
         <f>B43/C43</f>
-        <v>1.3333333333333333</v>
+        <v>0.26315789473684209</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="B44" s="3">
         <v>4</v>
       </c>
       <c r="C44" s="3">
-        <v>6</v>
-      </c>
-      <c r="D44" s="3">
+        <v>1</v>
+      </c>
+      <c r="D44" s="9">
         <f>B44/C44</f>
-        <v>0.66666666666666663</v>
+        <v>4</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>6</v>
@@ -1596,17 +1665,17 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="B45" s="3">
         <v>4</v>
       </c>
       <c r="C45" s="3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D45" s="3">
         <f>B45/C45</f>
-        <v>0.5</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>4</v>
@@ -1614,35 +1683,35 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="B46" s="3">
         <v>4</v>
       </c>
       <c r="C46" s="3">
-        <v>18</v>
-      </c>
-      <c r="D46" s="3">
+        <v>3</v>
+      </c>
+      <c r="D46" s="9">
         <f>B46/C46</f>
-        <v>0.22222222222222221</v>
+        <v>1.3333333333333333</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="B47" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" s="3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D47" s="3">
         <f>B47/C47</f>
-        <v>3</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>6</v>
@@ -1650,17 +1719,17 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="B48" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" s="3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D48" s="3">
         <f>B48/C48</f>
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>4</v>
@@ -1668,71 +1737,71 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B49" s="3">
         <v>3</v>
       </c>
       <c r="C49" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="3">
         <f>B49/C49</f>
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="B50" s="3">
         <v>3</v>
       </c>
       <c r="C50" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D50" s="3">
         <f>B50/C50</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>103</v>
+        <v>34</v>
       </c>
       <c r="B51" s="3">
         <v>3</v>
       </c>
       <c r="C51" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D51" s="3">
         <f>B51/C51</f>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="B52" s="3">
         <v>3</v>
       </c>
       <c r="C52" s="3">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D52" s="3">
         <f>B52/C52</f>
-        <v>0.375</v>
+        <v>0.6</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>9</v>
@@ -1740,115 +1809,115 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B53" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C53" s="3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D53" s="3">
         <f>B53/C53</f>
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="B54" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C54" s="3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D54" s="3">
         <f>B54/C54</f>
-        <v>2</v>
+        <v>0.375</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="B55" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C55" s="3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D55" s="3">
         <f>B55/C55</f>
-        <v>2</v>
+        <v>0.375</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="B56" s="3">
         <v>2</v>
       </c>
       <c r="C56" s="3">
-        <v>2</v>
-      </c>
-      <c r="D56" s="4">
+        <v>1</v>
+      </c>
+      <c r="D56" s="3">
         <f>B56/C56</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B57" s="3">
         <v>2</v>
       </c>
       <c r="C57" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" s="3">
         <f>B57/C57</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B58" s="3">
         <v>2</v>
       </c>
       <c r="C58" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" s="3">
         <f>B58/C58</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="B59" s="3">
         <v>2</v>
@@ -1856,7 +1925,7 @@
       <c r="C59" s="3">
         <v>2</v>
       </c>
-      <c r="D59" s="3">
+      <c r="D59" s="4">
         <f>B59/C59</f>
         <v>1</v>
       </c>
@@ -1866,7 +1935,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="B60" s="3">
         <v>2</v>
@@ -1879,76 +1948,76 @@
         <v>1</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B61" s="3">
         <v>2</v>
       </c>
       <c r="C61" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" s="3">
         <f>B61/C61</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B62" s="3">
         <v>2</v>
       </c>
       <c r="C62" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D62" s="3">
         <f>B62/C62</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B63" s="3">
         <v>2</v>
       </c>
       <c r="C63" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D63" s="3">
         <f>B63/C63</f>
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>106</v>
+        <v>32</v>
       </c>
       <c r="B64" s="3">
         <v>2</v>
       </c>
       <c r="C64" s="3">
-        <v>5</v>
-      </c>
-      <c r="D64" s="4">
+        <v>3</v>
+      </c>
+      <c r="D64" s="3">
         <f>B64/C64</f>
-        <v>0.4</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>9</v>
@@ -1956,35 +2025,35 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B65" s="3">
         <v>2</v>
       </c>
       <c r="C65" s="3">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D65" s="3">
         <f>B65/C65</f>
-        <v>0.2857142857142857</v>
+        <v>0.5</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="B66" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D66" s="3">
         <f>B66/C66</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>6</v>
@@ -1992,25 +2061,25 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>16</v>
+        <v>105</v>
       </c>
       <c r="B67" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" s="3">
-        <v>1</v>
-      </c>
-      <c r="D67" s="3">
+        <v>5</v>
+      </c>
+      <c r="D67" s="4">
         <f>B67/C67</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="B68" s="3">
         <v>1</v>
@@ -2028,7 +2097,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>107</v>
+        <v>16</v>
       </c>
       <c r="B69" s="3">
         <v>1</v>
@@ -2036,27 +2105,27 @@
       <c r="C69" s="3">
         <v>1</v>
       </c>
-      <c r="D69" s="4">
+      <c r="D69" s="3">
         <f>B69/C69</f>
         <v>1</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>108</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
-        <v>111</v>
+        <v>42</v>
       </c>
       <c r="B70" s="3">
         <v>1</v>
       </c>
       <c r="C70" s="3">
-        <v>2</v>
-      </c>
-      <c r="D70" s="9">
+        <v>1</v>
+      </c>
+      <c r="D70" s="3">
         <f>B70/C70</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>6</v>
@@ -2064,43 +2133,43 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="B71" s="3">
         <v>1</v>
       </c>
       <c r="C71" s="3">
-        <v>2</v>
-      </c>
-      <c r="D71" s="3">
+        <v>1</v>
+      </c>
+      <c r="D71" s="4">
         <f>B71/C71</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B72" s="3">
         <v>1</v>
       </c>
       <c r="C72" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D72" s="3">
         <f>B72/C72</f>
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
-        <v>94</v>
+        <v>30</v>
       </c>
       <c r="B73" s="3">
         <v>1</v>
@@ -2118,7 +2187,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B74" s="3">
         <v>1</v>
@@ -2131,22 +2200,22 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B75" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C75" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D75" s="3">
         <f>B75/C75</f>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>9</v>
@@ -2154,13 +2223,13 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B76" s="3">
         <v>0</v>
       </c>
       <c r="C76" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D76" s="3">
         <f>B76/C76</f>
@@ -2172,25 +2241,25 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="B77" s="3">
         <v>0</v>
       </c>
       <c r="C77" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D77" s="3">
         <f>B77/C77</f>
         <v>0</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B78" s="3">
         <v>0</v>
@@ -2208,7 +2277,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="B79" s="3">
         <v>0</v>
@@ -2221,48 +2290,48 @@
         <v>0</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="B80" s="3">
         <v>0</v>
       </c>
       <c r="C80" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D80" s="3">
         <f>B80/C80</f>
         <v>0</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="B81" s="3">
         <v>0</v>
       </c>
       <c r="C81" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D81" s="3">
         <f>B81/C81</f>
         <v>0</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="B82" s="3">
         <v>0</v>
@@ -2275,12 +2344,12 @@
         <v>0</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="B83" s="3">
         <v>0</v>
@@ -2298,7 +2367,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B84" s="3">
         <v>0</v>
@@ -2316,43 +2385,43 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="B85" s="3">
         <v>0</v>
       </c>
       <c r="C85" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D85" s="3">
         <f>B85/C85</f>
         <v>0</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="B86" s="3">
         <v>0</v>
       </c>
       <c r="C86" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="3">
         <f>B86/C86</f>
         <v>0</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B87" s="3">
         <v>0</v>
@@ -2365,12 +2434,12 @@
         <v>0</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B88" s="3">
         <v>0</v>
@@ -2383,12 +2452,12 @@
         <v>0</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="B89" s="3">
         <v>0</v>
@@ -2401,12 +2470,12 @@
         <v>0</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="B90" s="5">
         <v>0</v>
@@ -2419,12 +2488,12 @@
         <v>0</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="B91" s="5">
         <v>0</v>
@@ -2437,50 +2506,69 @@
         <v>0</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B92" s="5">
         <v>0</v>
       </c>
       <c r="C92" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D92" s="10">
+        <f>B92/C92</f>
         <v>0</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B93" s="6">
-        <v>0</v>
-      </c>
-      <c r="C93" s="6">
-        <v>0</v>
-      </c>
-      <c r="D93" s="7">
+        <v>89</v>
+      </c>
+      <c r="B93" s="5">
+        <v>0</v>
+      </c>
+      <c r="C93" s="5">
+        <v>0</v>
+      </c>
+      <c r="D93" s="10">
         <v>0</v>
       </c>
       <c r="E93" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B94" s="6">
+        <v>0</v>
+      </c>
+      <c r="C94" s="6">
+        <v>0</v>
+      </c>
+      <c r="D94" s="7">
+        <v>0</v>
+      </c>
+      <c r="E94" s="5" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E93">
-    <sortCondition descending="1" ref="B2:B93"/>
-    <sortCondition descending="1" ref="D2:D93"/>
-    <sortCondition descending="1" ref="C2:C93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E94">
+    <sortCondition descending="1" ref="B2:B94"/>
+    <sortCondition descending="1" ref="D2:D94"/>
+    <sortCondition descending="1" ref="C2:C94"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>